<commit_message>
Retrait de Christian Rémillard
</commit_message>
<xml_diff>
--- a/content/personnel/liste-personnel.xlsx
+++ b/content/personnel/liste-personnel.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="20417"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\projets\coquille-web\content\personnel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\p1196800\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F89B6ED4-F572-45E3-AC17-CAFADE094302}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1372C41-F016-4C85-82E4-B5567BDDFC56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="57840" windowHeight="31920" tabRatio="130" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="130" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,12 +20,23 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1090" uniqueCount="761">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1083" uniqueCount="758">
   <si>
     <t>nom</t>
   </si>
@@ -2106,9 +2117,6 @@
     <t>isabelle.giguere.4@umontreal.ca</t>
   </si>
   <si>
-    <t>christian.remillard@umontreal.ca</t>
-  </si>
-  <si>
     <t>stephanie.hainault@umontreal.ca</t>
   </si>
   <si>
@@ -2124,13 +2132,7 @@
     <t>Natalia</t>
   </si>
   <si>
-    <t>Webmestre</t>
-  </si>
-  <si>
     <t>Analyste en informatique</t>
-  </si>
-  <si>
-    <t>Rémillard</t>
   </si>
   <si>
     <t>Hainault</t>
@@ -2445,12 +2447,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="3">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -2461,10 +2462,10 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="2" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -2474,15 +2475,11 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="2"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
-  <cellStyles count="3">
+  <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" xr:uid="{00000000-000B-0000-0000-000008000000}"/>
-    <cellStyle name="Lien hypertexte" xfId="2" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="12">
@@ -2660,10 +2657,10 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4A0AF7E1-A614-44BF-8C48-5C26377DC552}" name="Tableau1" displayName="Tableau1" ref="A1:J143" totalsRowShown="0" headerRowDxfId="11" dataDxfId="10">
-  <autoFilter ref="A1:J143" xr:uid="{4A0AF7E1-A614-44BF-8C48-5C26377DC552}"/>
-  <sortState ref="A2:J143">
-    <sortCondition ref="A1:A143"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4A0AF7E1-A614-44BF-8C48-5C26377DC552}" name="Tableau1" displayName="Tableau1" ref="A1:J142" totalsRowShown="0" headerRowDxfId="11" dataDxfId="10">
+  <autoFilter ref="A1:J142" xr:uid="{4A0AF7E1-A614-44BF-8C48-5C26377DC552}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:J142">
+    <sortCondition ref="A1:A142"/>
   </sortState>
   <tableColumns count="10">
     <tableColumn id="1" xr3:uid="{4B04E1AF-0079-4AD2-81CA-E8A433733E21}" name="nom" dataDxfId="9"/>
@@ -2684,9 +2681,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Thème Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -2724,9 +2721,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -2759,26 +2756,9 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -2811,26 +2791,9 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -3004,22 +2967,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J143"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:J142"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="18.42578125" customWidth="1"/>
+    <col min="1" max="1" width="18.44140625" customWidth="1"/>
     <col min="2" max="2" width="13" customWidth="1"/>
-    <col min="3" max="3" width="33.85546875" customWidth="1"/>
-    <col min="4" max="4" width="45.28515625" customWidth="1"/>
-    <col min="5" max="5" width="58.140625" customWidth="1"/>
+    <col min="3" max="3" width="33.88671875" customWidth="1"/>
+    <col min="4" max="4" width="45.33203125" customWidth="1"/>
+    <col min="5" max="5" width="58.109375" customWidth="1"/>
     <col min="6" max="6" width="58" customWidth="1"/>
-    <col min="7" max="7" width="70.85546875" customWidth="1"/>
-    <col min="8" max="8" width="23.7109375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="41.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="86.5703125" customWidth="1"/>
+    <col min="7" max="7" width="70.88671875" customWidth="1"/>
+    <col min="8" max="8" width="23.6640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="41.44140625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="86.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3051,7 +3014,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2" s="5" t="s">
         <v>10</v>
       </c>
@@ -3082,7 +3045,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=alexandre.amar-zifkin@umontreal.ca</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
         <v>18</v>
       </c>
@@ -3113,16 +3076,16 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=viviane.angers@umontreal.ca</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>705</v>
+        <v>702</v>
       </c>
       <c r="B4" t="s">
-        <v>706</v>
+        <v>703</v>
       </c>
       <c r="C4" s="5"/>
       <c r="D4" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="E4" s="5" t="s">
         <v>76</v>
@@ -3134,14 +3097,14 @@
         <v>306</v>
       </c>
       <c r="I4" s="6" t="s">
-        <v>707</v>
+        <v>704</v>
       </c>
       <c r="J4" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=busch.antenor.alexandre@umontreal.ca</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5" s="5" t="s">
         <v>24</v>
       </c>
@@ -3172,7 +3135,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=nadege.arsa@bib.umontreal.ca</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" s="5" t="s">
         <v>32</v>
       </c>
@@ -3203,7 +3166,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=denis.arvisais@umontreal.ca</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A7" s="5" t="s">
         <v>38</v>
       </c>
@@ -3236,7 +3199,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=audrey.attia@umontreal.ca</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A8" s="5" t="s">
         <v>44</v>
       </c>
@@ -3258,14 +3221,14 @@
         <v>47</v>
       </c>
       <c r="I8" s="15" t="s">
-        <v>758</v>
+        <v>755</v>
       </c>
       <c r="J8" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=monica.audet@umontreal.ca</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>48</v>
       </c>
@@ -3295,7 +3258,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=valerie.bastien@umontreal.ca</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A10" s="5" t="s">
         <v>55</v>
       </c>
@@ -3323,7 +3286,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=magalie.beaudoin@umontreal.ca</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A11" s="5" t="s">
         <v>62</v>
       </c>
@@ -3356,7 +3319,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=maryna.beaulieu@umontreal.ca</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A12" s="5" t="s">
         <v>68</v>
       </c>
@@ -3367,7 +3330,7 @@
         <v>602</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>696</v>
+        <v>695</v>
       </c>
       <c r="E12" s="5" t="s">
         <v>69</v>
@@ -3376,7 +3339,7 @@
         <v>70</v>
       </c>
       <c r="G12" t="s">
-        <v>746</v>
+        <v>743</v>
       </c>
       <c r="H12" s="3" t="s">
         <v>71</v>
@@ -3389,7 +3352,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=audrey.begin-poissant@umontreal.ca</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>689</v>
       </c>
@@ -3397,7 +3360,7 @@
         <v>688</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>731</v>
+        <v>728</v>
       </c>
       <c r="D13" s="5" t="s">
         <v>27</v>
@@ -3420,7 +3383,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=nima.behforouz@umontreal.ca</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A14" s="5" t="s">
         <v>73</v>
       </c>
@@ -3450,36 +3413,35 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=christian.belanger@umontreal.ca</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A15" s="17" t="s">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A15" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="B15" s="17" t="s">
-        <v>752</v>
-      </c>
-      <c r="C15" s="17"/>
-      <c r="D15" s="17" t="s">
+      <c r="B15" s="5" t="s">
+        <v>749</v>
+      </c>
+      <c r="C15" s="5"/>
+      <c r="D15" s="5" t="s">
         <v>681</v>
       </c>
-      <c r="E15" s="17" t="s">
+      <c r="E15" s="5" t="s">
         <v>117</v>
       </c>
-      <c r="F15" s="18"/>
-      <c r="G15" s="17" t="s">
+      <c r="G15" s="5" t="s">
         <v>284</v>
       </c>
-      <c r="H15" s="19" t="s">
-        <v>753</v>
+      <c r="H15" s="3" t="s">
+        <v>750</v>
       </c>
       <c r="I15" s="6" t="s">
-        <v>754</v>
+        <v>751</v>
       </c>
       <c r="J15" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=billie.bergeron@umontreal.ca</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A16" s="5" t="s">
         <v>80</v>
       </c>
@@ -3512,7 +3474,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=amy.bergeron@umontreal.ca</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A17" s="5" t="s">
         <v>85</v>
       </c>
@@ -3541,7 +3503,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=amelie.bernard@umontreal.ca</v>
       </c>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A18" s="5" t="s">
         <v>90</v>
       </c>
@@ -3570,7 +3532,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=hugo.bernier@umontreal.ca</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>90</v>
       </c>
@@ -3597,7 +3559,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=marie-france.bernier@umontreal.ca</v>
       </c>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A20" s="5" t="s">
         <v>670</v>
       </c>
@@ -3628,7 +3590,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=cathy.bingoye@umontreal.ca</v>
       </c>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A21" s="5" t="s">
         <v>98</v>
       </c>
@@ -3659,16 +3621,16 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=simon.blais.longtin@umontreal.ca</v>
       </c>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>713</v>
+        <v>710</v>
       </c>
       <c r="B22" t="s">
-        <v>714</v>
+        <v>711</v>
       </c>
       <c r="C22" s="5"/>
       <c r="D22" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="E22" s="5" t="s">
         <v>76</v>
@@ -3677,14 +3639,14 @@
         <v>77</v>
       </c>
       <c r="I22" s="6" t="s">
-        <v>715</v>
+        <v>712</v>
       </c>
       <c r="J22" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=guy.blondeau@umontreal.ca</v>
       </c>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>104</v>
       </c>
@@ -3714,7 +3676,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=tatiana.talpa@umontreal.ca</v>
       </c>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A24" s="3" t="s">
         <v>110</v>
       </c>
@@ -3740,7 +3702,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=joanna.bodnar@umontreal.ca</v>
       </c>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A25" s="5" t="s">
         <v>114</v>
       </c>
@@ -3770,7 +3732,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=alain.borsi@umontreal.ca</v>
       </c>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A26" s="5" t="s">
         <v>121</v>
       </c>
@@ -3801,7 +3763,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=eric.p.bouchard@umontreal.ca</v>
       </c>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A27" s="5" t="s">
         <v>128</v>
       </c>
@@ -3832,7 +3794,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=refdroi@bib.umontreal.ca</v>
       </c>
     </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A28" s="5" t="s">
         <v>134</v>
       </c>
@@ -3852,7 +3814,7 @@
         <v>598</v>
       </c>
       <c r="G28" s="5" t="s">
-        <v>747</v>
+        <v>744</v>
       </c>
       <c r="H28" s="5" t="s">
         <v>136</v>
@@ -3865,7 +3827,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=myriam.boyer@umontreal.ca</v>
       </c>
     </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A29" s="5" t="s">
         <v>138</v>
       </c>
@@ -3885,7 +3847,7 @@
         <v>346</v>
       </c>
       <c r="G29" s="5" t="s">
-        <v>747</v>
+        <v>744</v>
       </c>
       <c r="H29" s="5" t="s">
         <v>140</v>
@@ -3898,7 +3860,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=guylaine.brazeau@umontreal.ca</v>
       </c>
     </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A30" s="5" t="s">
         <v>675</v>
       </c>
@@ -3906,7 +3868,7 @@
         <v>344</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>744</v>
+        <v>741</v>
       </c>
       <c r="D30" s="5" t="s">
         <v>678</v>
@@ -3927,7 +3889,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=anne-marie.brien.1@umontreal.ca</v>
       </c>
     </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A31" s="5" t="s">
         <v>142</v>
       </c>
@@ -3955,7 +3917,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=sophie.brisebois@umontreal.ca</v>
       </c>
     </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A32" s="5" t="s">
         <v>657</v>
       </c>
@@ -3988,7 +3950,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=tanya.buchet@umontreal.ca</v>
       </c>
     </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>147</v>
       </c>
@@ -4015,16 +3977,16 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=fanny.c.brochu@umontreal.ca</v>
       </c>
     </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>722</v>
+        <v>719</v>
       </c>
       <c r="B34" t="s">
-        <v>723</v>
+        <v>720</v>
       </c>
       <c r="C34" s="5"/>
       <c r="D34" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="E34" s="5" t="s">
         <v>76</v>
@@ -4033,17 +3995,17 @@
         <v>77</v>
       </c>
       <c r="H34" t="s">
-        <v>720</v>
+        <v>717</v>
       </c>
       <c r="I34" s="6" t="s">
-        <v>724</v>
+        <v>721</v>
       </c>
       <c r="J34" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=thierry.caballero@umontreal.ca</v>
       </c>
     </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A35" s="5" t="s">
         <v>151</v>
       </c>
@@ -4060,7 +4022,7 @@
         <v>117</v>
       </c>
       <c r="F35" t="s">
-        <v>743</v>
+        <v>740</v>
       </c>
       <c r="G35" s="5" t="s">
         <v>154</v>
@@ -4076,7 +4038,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=delphine.cado@umontreal.ca</v>
       </c>
     </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A36" s="5" t="s">
         <v>157</v>
       </c>
@@ -4105,7 +4067,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=siv.kham.chao@umontreal.ca</v>
       </c>
     </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A37" s="5" t="s">
         <v>162</v>
       </c>
@@ -4136,7 +4098,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=laurence.charest@umontreal.ca</v>
       </c>
     </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>169</v>
       </c>
@@ -4160,16 +4122,16 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=annick.charette@umontreal.ca</v>
       </c>
     </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>725</v>
+        <v>722</v>
       </c>
       <c r="B39" t="s">
-        <v>726</v>
+        <v>723</v>
       </c>
       <c r="C39" s="5"/>
       <c r="D39" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="E39" s="5" t="s">
         <v>76</v>
@@ -4178,17 +4140,17 @@
         <v>77</v>
       </c>
       <c r="H39" t="s">
-        <v>720</v>
+        <v>717</v>
       </c>
       <c r="I39" t="s">
-        <v>727</v>
+        <v>724</v>
       </c>
       <c r="J39" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=wassif.cheikh@umontreal.ca</v>
       </c>
     </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A40" s="5" t="s">
         <v>173</v>
       </c>
@@ -4216,7 +4178,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=mailto:thien-huong.che-quang@umontreal.ca</v>
       </c>
     </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A41" s="5" t="s">
         <v>175</v>
       </c>
@@ -4247,7 +4209,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=sarah.cherrier@umontreal.ca</v>
       </c>
     </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A42" s="5" t="s">
         <v>181</v>
       </c>
@@ -4277,7 +4239,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=emir.chouchane@umontreal.ca</v>
       </c>
     </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A43" s="5" t="s">
         <v>187</v>
       </c>
@@ -4308,7 +4270,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=accessibilite@bib.umontreal.ca</v>
       </c>
     </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A44" s="5" t="s">
         <v>192</v>
       </c>
@@ -4341,7 +4303,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=benjamin.constantineau@umontreal.ca</v>
       </c>
     </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A45" s="5" t="s">
         <v>199</v>
       </c>
@@ -4372,7 +4334,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=simon-pierre.crevier@umontreal.ca</v>
       </c>
     </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A46" s="5" t="s">
         <v>205</v>
       </c>
@@ -4387,7 +4349,7 @@
       </c>
       <c r="E46" s="5"/>
       <c r="F46" s="5" t="s">
-        <v>745</v>
+        <v>742</v>
       </c>
       <c r="G46" s="5" t="s">
         <v>52</v>
@@ -4403,7 +4365,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=marc-olivier.croteau@umontreal.ca</v>
       </c>
     </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A47" s="5" t="s">
         <v>209</v>
       </c>
@@ -4434,7 +4396,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=emilie.dalpe@umontreal.ca</v>
       </c>
     </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A48" s="5" t="s">
         <v>215</v>
       </c>
@@ -4465,7 +4427,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=morgane.de.bellefeuille@umontreal.ca</v>
       </c>
     </row>
-    <row r="49" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A49" s="5" t="s">
         <v>222</v>
       </c>
@@ -4496,7 +4458,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=Indiana.delsart@umontreal.ca</v>
       </c>
     </row>
-    <row r="50" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A50" s="5" t="s">
         <v>228</v>
       </c>
@@ -4527,7 +4489,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=dominic.desaulniers@umontreal.ca</v>
       </c>
     </row>
-    <row r="51" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A51" s="5" t="s">
         <v>234</v>
       </c>
@@ -4556,7 +4518,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=chantal.desrosiers@umontreal.ca</v>
       </c>
     </row>
-    <row r="52" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>239</v>
       </c>
@@ -4583,7 +4545,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=anne.dubois.mercier@umontreal.ca</v>
       </c>
     </row>
-    <row r="53" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A53" s="5" t="s">
         <v>243</v>
       </c>
@@ -4614,7 +4576,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=jean-francois.durnin@umontreal.ca</v>
       </c>
     </row>
-    <row r="54" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A54" s="5" t="s">
         <v>652</v>
       </c>
@@ -4645,7 +4607,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=taline.ekmekjian@umontreal.ca</v>
       </c>
     </row>
-    <row r="55" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>249</v>
       </c>
@@ -4672,7 +4634,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=judith.fafard-larose@umontreal.ca</v>
       </c>
     </row>
-    <row r="56" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A56" s="5" t="s">
         <v>253</v>
       </c>
@@ -4705,7 +4667,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=sylvie.fontaine.1@umontreal.ca</v>
       </c>
     </row>
-    <row r="57" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A57" s="5" t="s">
         <v>258</v>
       </c>
@@ -4738,7 +4700,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=c.fortier@umontreal.ca</v>
       </c>
     </row>
-    <row r="58" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A58" s="5" t="s">
         <v>264</v>
       </c>
@@ -4765,7 +4727,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=7077duParc@bib.umontreal.ca</v>
       </c>
     </row>
-    <row r="59" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A59" s="5" t="s">
         <v>270</v>
       </c>
@@ -4796,7 +4758,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=nino.gabrielli@umontreal.ca</v>
       </c>
     </row>
-    <row r="60" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A60" s="5" t="s">
         <v>276</v>
       </c>
@@ -4825,7 +4787,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=marie-pierre.gadoua@umontreal.ca</v>
       </c>
     </row>
-    <row r="61" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A61" s="5" t="s">
         <v>280</v>
       </c>
@@ -4856,7 +4818,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=cynthia.gagne.2@umontreal.ca</v>
       </c>
     </row>
-    <row r="62" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A62" s="5" t="s">
         <v>287</v>
       </c>
@@ -4882,7 +4844,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=diane.gagnon@umontreal.ca</v>
       </c>
     </row>
-    <row r="63" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A63" s="5" t="s">
         <v>287</v>
       </c>
@@ -4910,7 +4872,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=stephanie.gagnon@umontreal.ca</v>
       </c>
     </row>
-    <row r="64" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A64" s="5" t="s">
         <v>293</v>
       </c>
@@ -4940,12 +4902,12 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=marjorie.gauchier@umontreal.ca</v>
       </c>
     </row>
-    <row r="65" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
-        <v>704</v>
+        <v>701</v>
       </c>
       <c r="B65" t="s">
-        <v>697</v>
+        <v>696</v>
       </c>
       <c r="C65" s="5"/>
       <c r="D65" s="5" t="s">
@@ -4969,7 +4931,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=lucie.geoffroy@umontreal.ca</v>
       </c>
     </row>
-    <row r="66" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A66" s="5" t="s">
         <v>299</v>
       </c>
@@ -4996,7 +4958,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=noemie.gervais@umontreal.ca</v>
       </c>
     </row>
-    <row r="67" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A67" s="5" t="s">
         <v>302</v>
       </c>
@@ -5029,18 +4991,18 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=isabelle.giguere.4@umontreal.ca</v>
       </c>
     </row>
-    <row r="68" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
-        <v>702</v>
+        <v>699</v>
       </c>
       <c r="B68" t="s">
         <v>288</v>
       </c>
       <c r="C68" s="5" t="s">
-        <v>730</v>
+        <v>727</v>
       </c>
       <c r="D68" t="s">
-        <v>696</v>
+        <v>695</v>
       </c>
       <c r="E68" s="5" t="s">
         <v>76</v>
@@ -5053,14 +5015,14 @@
         <v>306</v>
       </c>
       <c r="I68" t="s">
-        <v>694</v>
+        <v>693</v>
       </c>
       <c r="J68" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=stephanie.hainault@umontreal.ca</v>
       </c>
     </row>
-    <row r="69" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A69" s="5" t="s">
         <v>307</v>
       </c>
@@ -5091,7 +5053,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=anne.hakier@umontreal.ca</v>
       </c>
     </row>
-    <row r="70" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A70" s="5" t="s">
         <v>312</v>
       </c>
@@ -5122,7 +5084,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=rose.carine.henriquez@umontreal.ca</v>
       </c>
     </row>
-    <row r="71" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
         <v>318</v>
       </c>
@@ -5152,18 +5114,18 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=thien.sa.hoang@umontreal.ca</v>
       </c>
     </row>
-    <row r="72" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
-        <v>703</v>
+        <v>700</v>
       </c>
       <c r="B72" t="s">
+        <v>697</v>
+      </c>
+      <c r="C72" s="5" t="s">
+        <v>729</v>
+      </c>
+      <c r="D72" t="s">
         <v>698</v>
-      </c>
-      <c r="C72" s="5" t="s">
-        <v>732</v>
-      </c>
-      <c r="D72" t="s">
-        <v>700</v>
       </c>
       <c r="E72" s="5" t="s">
         <v>76</v>
@@ -5176,14 +5138,14 @@
         <v>306</v>
       </c>
       <c r="I72" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
       <c r="J72" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=natalia.jabinschi@umontreal.ca</v>
       </c>
     </row>
-    <row r="73" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A73" s="5" t="s">
         <v>324</v>
       </c>
@@ -5212,7 +5174,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=khalid.jouamaa@umontreal.ca</v>
       </c>
     </row>
-    <row r="74" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A74" s="5" t="s">
         <v>329</v>
       </c>
@@ -5243,7 +5205,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=aminata.keita@umontreal.ca</v>
       </c>
     </row>
-    <row r="75" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
         <v>334</v>
       </c>
@@ -5270,16 +5232,16 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=melanie.lachapelle@umontreal.ca</v>
       </c>
     </row>
-    <row r="76" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
-        <v>708</v>
+        <v>705</v>
       </c>
       <c r="B76" t="s">
-        <v>709</v>
+        <v>706</v>
       </c>
       <c r="C76" s="5"/>
       <c r="D76" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="E76" s="5" t="s">
         <v>76</v>
@@ -5292,14 +5254,14 @@
         <v>306</v>
       </c>
       <c r="I76" s="6" t="s">
-        <v>710</v>
+        <v>707</v>
       </c>
       <c r="J76" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=pierre-yves.lafleur@umontreal.ca</v>
       </c>
     </row>
-    <row r="77" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A77" s="5" t="s">
         <v>338</v>
       </c>
@@ -5326,7 +5288,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=isabelle.lagadec@umontreal.ca</v>
       </c>
     </row>
-    <row r="78" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
         <v>340</v>
       </c>
@@ -5353,7 +5315,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=marie-france.laliberte@umontreal.ca</v>
       </c>
     </row>
-    <row r="79" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A79" s="5" t="s">
         <v>343</v>
       </c>
@@ -5373,7 +5335,7 @@
         <v>346</v>
       </c>
       <c r="G79" s="5" t="s">
-        <v>747</v>
+        <v>744</v>
       </c>
       <c r="H79" s="5" t="s">
         <v>347</v>
@@ -5386,7 +5348,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=am.lalonde@umontreal.ca</v>
       </c>
     </row>
-    <row r="80" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A80" s="5" t="s">
         <v>349</v>
       </c>
@@ -5419,16 +5381,16 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=tara.landry@umontreal.ca</v>
       </c>
     </row>
-    <row r="81" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A81" s="5" t="s">
-        <v>733</v>
+        <v>730</v>
       </c>
       <c r="B81" s="5" t="s">
-        <v>734</v>
+        <v>731</v>
       </c>
       <c r="C81" s="5"/>
       <c r="D81" s="5" t="s">
-        <v>735</v>
+        <v>732</v>
       </c>
       <c r="E81" s="5" t="s">
         <v>641</v>
@@ -5438,17 +5400,17 @@
         <v>125</v>
       </c>
       <c r="H81" s="5" t="s">
-        <v>736</v>
+        <v>733</v>
       </c>
       <c r="I81" s="6" t="s">
-        <v>737</v>
+        <v>734</v>
       </c>
       <c r="J81" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=marie-josee.lapalme@umontreal.ca</v>
       </c>
     </row>
-    <row r="82" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A82" s="5" t="s">
         <v>354</v>
       </c>
@@ -5481,7 +5443,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=stephanie.lariviere-roberge@umontreal.ca</v>
       </c>
     </row>
-    <row r="83" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
         <v>358</v>
       </c>
@@ -5508,7 +5470,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=alex-sandrine.lavallee-masse@umontreal.ca</v>
       </c>
     </row>
-    <row r="84" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A84" s="5" t="s">
         <v>362</v>
       </c>
@@ -5539,7 +5501,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=graham.lavender@umontreal.ca</v>
       </c>
     </row>
-    <row r="85" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
         <v>367</v>
       </c>
@@ -5556,7 +5518,7 @@
         <v>69</v>
       </c>
       <c r="F85" t="s">
-        <v>748</v>
+        <v>745</v>
       </c>
       <c r="G85" s="5" t="s">
         <v>424</v>
@@ -5572,7 +5534,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=jessica.legault.2@umontreal.ca</v>
       </c>
     </row>
-    <row r="86" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A86" s="5" t="s">
         <v>371</v>
       </c>
@@ -5603,7 +5565,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=genevieve.lemarier@umontreal.ca</v>
       </c>
     </row>
-    <row r="87" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A87" s="5" t="s">
         <v>376</v>
       </c>
@@ -5636,7 +5598,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=mariane.leonard@umontreal.ca</v>
       </c>
     </row>
-    <row r="88" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A88" s="5" t="s">
         <v>382</v>
       </c>
@@ -5666,7 +5628,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=maude.lethiecq-normand@umontreal.ca</v>
       </c>
     </row>
-    <row r="89" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A89" s="5" t="s">
         <v>386</v>
       </c>
@@ -5697,7 +5659,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=danny.letourneau@umontreal.ca</v>
       </c>
     </row>
-    <row r="90" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A90" s="3" t="s">
         <v>391</v>
       </c>
@@ -5730,7 +5692,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=ae.levesque@umontreal.ca</v>
       </c>
     </row>
-    <row r="91" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A91" s="5" t="s">
         <v>391</v>
       </c>
@@ -5756,7 +5718,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=anny.levesque@umontreal.ca</v>
       </c>
     </row>
-    <row r="92" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A92" s="5" t="s">
         <v>397</v>
       </c>
@@ -5785,7 +5747,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=jason.madooray@umontreal.ca</v>
       </c>
     </row>
-    <row r="93" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A93" s="5" t="s">
         <v>401</v>
       </c>
@@ -5814,7 +5776,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=yacine.mansar@umontreal.ca</v>
       </c>
     </row>
-    <row r="94" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A94" s="5" t="s">
         <v>406</v>
       </c>
@@ -5842,7 +5804,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=vanessa.martin.2@umontreal.ca</v>
       </c>
     </row>
-    <row r="95" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A95" s="5" t="s">
         <v>410</v>
       </c>
@@ -5873,7 +5835,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=pascal.martinolli@umontreal.ca</v>
       </c>
     </row>
-    <row r="96" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A96" s="5" t="s">
         <v>415</v>
       </c>
@@ -5904,7 +5866,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=melanie.masse.2@umontreal.ca</v>
       </c>
     </row>
-    <row r="97" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A97" s="5" t="s">
         <v>421</v>
       </c>
@@ -5934,7 +5896,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=gabrielle.mathieu-dupuis@umontreal.ca</v>
       </c>
     </row>
-    <row r="98" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A98" s="5" t="s">
         <v>427</v>
       </c>
@@ -5963,7 +5925,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=benoit.mayrand@umontreal.ca</v>
       </c>
     </row>
-    <row r="99" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A99" s="5" t="s">
         <v>431</v>
       </c>
@@ -5994,7 +5956,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=christiane.melancon@umontreal.ca</v>
       </c>
     </row>
-    <row r="100" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A100" s="3" t="s">
         <v>437</v>
       </c>
@@ -6025,7 +5987,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=ginette-denyse.melancon.bolduc@umontreal.ca</v>
       </c>
     </row>
-    <row r="101" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A101" s="5" t="s">
         <v>442</v>
       </c>
@@ -6042,10 +6004,10 @@
         <v>69</v>
       </c>
       <c r="F101" s="5" t="s">
-        <v>749</v>
+        <v>746</v>
       </c>
       <c r="G101" s="5" t="s">
-        <v>746</v>
+        <v>743</v>
       </c>
       <c r="H101" s="5" t="s">
         <v>445</v>
@@ -6058,15 +6020,15 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=justine.menard.1@umontreal.ca</v>
       </c>
     </row>
-    <row r="102" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A102" s="5" t="s">
-        <v>738</v>
+        <v>735</v>
       </c>
       <c r="B102" s="5" t="s">
         <v>291</v>
       </c>
       <c r="C102" s="5" t="s">
-        <v>739</v>
+        <v>736</v>
       </c>
       <c r="D102" s="5" t="s">
         <v>678</v>
@@ -6079,17 +6041,17 @@
         <v>125</v>
       </c>
       <c r="H102" s="5" t="s">
-        <v>740</v>
+        <v>737</v>
       </c>
       <c r="I102" s="6" t="s">
-        <v>741</v>
+        <v>738</v>
       </c>
       <c r="J102" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=diane.moreau@umontreal.ca</v>
       </c>
     </row>
-    <row r="103" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A103" t="s">
         <v>447</v>
       </c>
@@ -6106,7 +6068,7 @@
         <v>69</v>
       </c>
       <c r="F103" t="s">
-        <v>750</v>
+        <v>747</v>
       </c>
       <c r="G103" s="5" t="s">
         <v>424</v>
@@ -6122,7 +6084,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=mathieu.murray-samuel@umontreal.ca</v>
       </c>
     </row>
-    <row r="104" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A104" s="3" t="s">
         <v>451</v>
       </c>
@@ -6153,7 +6115,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=france.nadeau@umontreal.ca</v>
       </c>
     </row>
-    <row r="105" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A105" s="5" t="s">
         <v>455</v>
       </c>
@@ -6184,7 +6146,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=magdalena.oriental@umontreal.ca</v>
       </c>
     </row>
-    <row r="106" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A106" s="5" t="s">
         <v>461</v>
       </c>
@@ -6210,7 +6172,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=fatima.zahra.ouadrhiri@umontreal.ca</v>
       </c>
     </row>
-    <row r="107" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A107" s="5" t="s">
         <v>465</v>
       </c>
@@ -6224,11 +6186,11 @@
         <v>683</v>
       </c>
       <c r="E107" t="s">
-        <v>759</v>
+        <v>756</v>
       </c>
       <c r="F107" s="3"/>
       <c r="G107" t="s">
-        <v>755</v>
+        <v>752</v>
       </c>
       <c r="H107" s="5" t="s">
         <v>467</v>
@@ -6241,7 +6203,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=julie.ouellette@umontreal.ca</v>
       </c>
     </row>
-    <row r="108" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A108" s="5" t="s">
         <v>469</v>
       </c>
@@ -6250,11 +6212,11 @@
       </c>
       <c r="C108" s="5"/>
       <c r="D108" s="5" t="s">
-        <v>756</v>
-      </c>
-      <c r="E108" s="17"/>
+        <v>753</v>
+      </c>
+      <c r="E108" s="5"/>
       <c r="G108" s="5" t="s">
-        <v>760</v>
+        <v>757</v>
       </c>
       <c r="H108" s="5"/>
       <c r="I108" s="8" t="s">
@@ -6265,7 +6227,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=francois-xavier.panaccio@umontreal.ca</v>
       </c>
     </row>
-    <row r="109" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A109" s="5" t="s">
         <v>473</v>
       </c>
@@ -6296,7 +6258,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=caroline.patenaude@umontreal.ca</v>
       </c>
     </row>
-    <row r="110" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A110" s="5" t="s">
         <v>473</v>
       </c>
@@ -6329,7 +6291,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=david.patenaude.1@umontreal.ca</v>
       </c>
     </row>
-    <row r="111" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A111" s="5" t="s">
         <v>482</v>
       </c>
@@ -6360,7 +6322,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=stephanie.pham-dang@umontreal.ca</v>
       </c>
     </row>
-    <row r="112" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A112" s="5" t="s">
         <v>486</v>
       </c>
@@ -6389,7 +6351,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=mathieu.pigeon@umontreal.ca</v>
       </c>
     </row>
-    <row r="113" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A113" s="5" t="s">
         <v>490</v>
       </c>
@@ -6420,7 +6382,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=refmede@bib.umontreal.ca</v>
       </c>
     </row>
-    <row r="114" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A114" s="5" t="s">
         <v>496</v>
       </c>
@@ -6449,7 +6411,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=nathalie.poulin.4@umontreal.ca</v>
       </c>
     </row>
-    <row r="115" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A115" t="s">
         <v>500</v>
       </c>
@@ -6476,16 +6438,16 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=jeremy.prime@umontreal.ca</v>
       </c>
     </row>
-    <row r="116" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A116" t="s">
-        <v>711</v>
+        <v>708</v>
       </c>
       <c r="B116" t="s">
         <v>448</v>
       </c>
       <c r="C116" s="14"/>
       <c r="D116" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="E116" s="5" t="s">
         <v>76</v>
@@ -6497,14 +6459,14 @@
         <v>306</v>
       </c>
       <c r="I116" s="6" t="s">
-        <v>712</v>
+        <v>709</v>
       </c>
       <c r="J116" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=mathieu.proulx@umontreal.ca</v>
       </c>
     </row>
-    <row r="117" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A117" t="s">
         <v>504</v>
       </c>
@@ -6529,596 +6491,596 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=clotilde.rajalu@umontreal.ca</v>
       </c>
     </row>
-    <row r="118" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A118" t="s">
-        <v>701</v>
+        <v>639</v>
       </c>
       <c r="B118" t="s">
-        <v>74</v>
-      </c>
-      <c r="C118" s="5"/>
-      <c r="D118" t="s">
-        <v>699</v>
-      </c>
-      <c r="E118" s="5" t="s">
+        <v>640</v>
+      </c>
+      <c r="C118" s="5" t="s">
+        <v>648</v>
+      </c>
+      <c r="D118" s="5" t="s">
+        <v>678</v>
+      </c>
+      <c r="E118" s="5"/>
+      <c r="F118" s="3"/>
+      <c r="G118" t="s">
+        <v>525</v>
+      </c>
+      <c r="H118" t="s">
+        <v>642</v>
+      </c>
+      <c r="I118" s="6" t="s">
+        <v>643</v>
+      </c>
+      <c r="J118" s="6" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=sarah-julie.richard@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="119" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A119" t="s">
+        <v>508</v>
+      </c>
+      <c r="B119" t="s">
+        <v>49</v>
+      </c>
+      <c r="C119" s="7" t="s">
+        <v>509</v>
+      </c>
+      <c r="D119" t="s">
+        <v>13</v>
+      </c>
+      <c r="F119" s="5" t="s">
+        <v>510</v>
+      </c>
+      <c r="G119" t="s">
+        <v>29</v>
+      </c>
+      <c r="H119" s="3" t="s">
+        <v>511</v>
+      </c>
+      <c r="I119" s="3" t="s">
+        <v>512</v>
+      </c>
+      <c r="J119" s="6" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=valerie.rioux.3@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="120" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A120" t="s">
+        <v>716</v>
+      </c>
+      <c r="B120" t="s">
+        <v>122</v>
+      </c>
+      <c r="C120" s="5"/>
+      <c r="D120" t="s">
+        <v>725</v>
+      </c>
+      <c r="E120" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="F118" s="5"/>
-      <c r="G118" s="5" t="s">
-        <v>305</v>
-      </c>
-      <c r="H118" s="5" t="s">
-        <v>306</v>
-      </c>
-      <c r="I118" t="s">
-        <v>693</v>
-      </c>
-      <c r="J118" s="9" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=christian.remillard@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="119" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A119" t="s">
-        <v>639</v>
-      </c>
-      <c r="B119" t="s">
-        <v>640</v>
-      </c>
-      <c r="C119" s="5" t="s">
-        <v>648</v>
-      </c>
-      <c r="D119" s="5" t="s">
-        <v>678</v>
-      </c>
-      <c r="E119" s="5"/>
-      <c r="F119" s="3"/>
-      <c r="G119" t="s">
-        <v>525</v>
-      </c>
-      <c r="H119" t="s">
-        <v>642</v>
-      </c>
-      <c r="I119" s="6" t="s">
-        <v>643</v>
-      </c>
-      <c r="J119" s="6" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=sarah-julie.richard@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="120" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A120" t="s">
-        <v>508</v>
-      </c>
-      <c r="B120" t="s">
-        <v>49</v>
-      </c>
-      <c r="C120" s="7" t="s">
-        <v>509</v>
-      </c>
-      <c r="D120" t="s">
-        <v>13</v>
-      </c>
-      <c r="F120" s="5" t="s">
-        <v>510</v>
-      </c>
       <c r="G120" t="s">
-        <v>29</v>
-      </c>
-      <c r="H120" s="3" t="s">
-        <v>511</v>
-      </c>
-      <c r="I120" s="3" t="s">
-        <v>512</v>
-      </c>
-      <c r="J120" s="6" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=valerie.rioux.3@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="121" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A121" t="s">
-        <v>719</v>
-      </c>
-      <c r="B121" t="s">
-        <v>122</v>
-      </c>
-      <c r="C121" s="5"/>
-      <c r="D121" t="s">
-        <v>728</v>
+        <v>77</v>
+      </c>
+      <c r="H120" t="s">
+        <v>717</v>
+      </c>
+      <c r="I120" s="6" t="s">
+        <v>718</v>
+      </c>
+      <c r="J120" s="9" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=eric.romano@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="121" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A121" s="5" t="s">
+        <v>513</v>
+      </c>
+      <c r="B121" s="5" t="s">
+        <v>406</v>
+      </c>
+      <c r="C121" s="5" t="s">
+        <v>514</v>
+      </c>
+      <c r="D121" s="5" t="s">
+        <v>684</v>
       </c>
       <c r="E121" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="G121" t="s">
-        <v>77</v>
-      </c>
-      <c r="H121" t="s">
-        <v>720</v>
-      </c>
-      <c r="I121" s="6" t="s">
-        <v>721</v>
-      </c>
-      <c r="J121" s="9" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=eric.romano@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="122" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="F121" s="5"/>
+      <c r="H121" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="I121" s="15" t="s">
+        <v>515</v>
+      </c>
+      <c r="J121" s="6" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=m.sevigny@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="122" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A122" s="5" t="s">
-        <v>513</v>
+        <v>516</v>
       </c>
       <c r="B122" s="5" t="s">
-        <v>406</v>
+        <v>517</v>
       </c>
       <c r="C122" s="5" t="s">
-        <v>514</v>
+        <v>606</v>
       </c>
       <c r="D122" s="5" t="s">
-        <v>684</v>
-      </c>
-      <c r="E122" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E122" s="5"/>
+      <c r="F122" s="5" t="s">
+        <v>518</v>
+      </c>
+      <c r="G122" s="5" t="s">
+        <v>154</v>
+      </c>
+      <c r="H122" s="3"/>
+      <c r="I122" s="3" t="s">
+        <v>519</v>
+      </c>
+      <c r="J122" s="6" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=chloe.sinotte@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="123" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A123" t="s">
+        <v>520</v>
+      </c>
+      <c r="B123" t="s">
+        <v>521</v>
+      </c>
+      <c r="C123" t="s">
+        <v>601</v>
+      </c>
+      <c r="D123" s="3" t="s">
+        <v>679</v>
+      </c>
+      <c r="E123" s="5"/>
+      <c r="F123" s="5"/>
+      <c r="G123" t="s">
+        <v>29</v>
+      </c>
+      <c r="J123" s="6" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="124" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A124" s="3" t="s">
+        <v>522</v>
+      </c>
+      <c r="B124" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C124" s="14" t="s">
+        <v>523</v>
+      </c>
+      <c r="D124" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="E124" s="3"/>
+      <c r="F124" s="3" t="s">
+        <v>524</v>
+      </c>
+      <c r="G124" s="3" t="s">
+        <v>525</v>
+      </c>
+      <c r="H124" s="3" t="s">
+        <v>526</v>
+      </c>
+      <c r="I124" s="3" t="s">
+        <v>527</v>
+      </c>
+      <c r="J124" s="6" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=viviane.st-arnaud@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="125" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A125" s="3" t="s">
+        <v>528</v>
+      </c>
+      <c r="B125" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="C125" s="3"/>
+      <c r="D125" s="3" t="s">
+        <v>679</v>
+      </c>
+      <c r="E125" s="3" t="s">
+        <v>542</v>
+      </c>
+      <c r="F125" s="3"/>
+      <c r="G125" s="3" t="s">
+        <v>754</v>
+      </c>
+      <c r="H125" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="I125" s="3" t="s">
+        <v>530</v>
+      </c>
+      <c r="J125" s="6" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=chantal.taillon@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="126" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A126" s="5" t="s">
+        <v>531</v>
+      </c>
+      <c r="B126" s="5" t="s">
+        <v>532</v>
+      </c>
+      <c r="C126" s="5" t="s">
+        <v>533</v>
+      </c>
+      <c r="D126" s="5" t="s">
+        <v>683</v>
+      </c>
+      <c r="E126" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="F122" s="5"/>
-      <c r="H122" s="3" t="s">
-        <v>112</v>
-      </c>
-      <c r="I122" s="15" t="s">
-        <v>515</v>
-      </c>
-      <c r="J122" s="6" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=m.sevigny@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="123" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A123" s="5" t="s">
-        <v>516</v>
-      </c>
-      <c r="B123" s="5" t="s">
-        <v>517</v>
-      </c>
-      <c r="C123" s="5" t="s">
-        <v>606</v>
-      </c>
-      <c r="D123" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="E123" s="5"/>
-      <c r="F123" s="5" t="s">
-        <v>518</v>
-      </c>
-      <c r="G123" s="5" t="s">
-        <v>154</v>
-      </c>
-      <c r="H123" s="3"/>
-      <c r="I123" s="3" t="s">
-        <v>519</v>
-      </c>
-      <c r="J123" s="6" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=chloe.sinotte@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="124" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A124" t="s">
-        <v>520</v>
-      </c>
-      <c r="B124" t="s">
-        <v>521</v>
-      </c>
-      <c r="C124" t="s">
-        <v>601</v>
-      </c>
-      <c r="D124" s="3" t="s">
-        <v>679</v>
-      </c>
-      <c r="E124" s="5"/>
-      <c r="F124" s="5"/>
-      <c r="G124" t="s">
-        <v>29</v>
-      </c>
-      <c r="J124" s="6" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="125" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A125" s="3" t="s">
-        <v>522</v>
-      </c>
-      <c r="B125" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="C125" s="14" t="s">
-        <v>523</v>
-      </c>
-      <c r="D125" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="E125" s="3"/>
-      <c r="F125" s="3" t="s">
-        <v>524</v>
-      </c>
-      <c r="G125" s="3" t="s">
+      <c r="G126" s="5" t="s">
+        <v>305</v>
+      </c>
+      <c r="H126" s="5" t="s">
+        <v>534</v>
+      </c>
+      <c r="I126" s="15" t="s">
+        <v>535</v>
+      </c>
+      <c r="J126" s="6" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=mathieu.nicolas.tardif@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="127" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A127" t="s">
+        <v>644</v>
+      </c>
+      <c r="B127" t="s">
+        <v>566</v>
+      </c>
+      <c r="C127" s="5" t="s">
+        <v>647</v>
+      </c>
+      <c r="D127" s="5" t="s">
+        <v>678</v>
+      </c>
+      <c r="E127" s="5"/>
+      <c r="F127" s="3"/>
+      <c r="G127" t="s">
         <v>525</v>
       </c>
-      <c r="H125" s="3" t="s">
-        <v>526</v>
-      </c>
-      <c r="I125" s="3" t="s">
-        <v>527</v>
-      </c>
-      <c r="J125" s="6" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=viviane.st-arnaud@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="126" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A126" s="3" t="s">
-        <v>528</v>
-      </c>
-      <c r="B126" s="3" t="s">
-        <v>235</v>
-      </c>
-      <c r="C126" s="3"/>
-      <c r="D126" s="3" t="s">
-        <v>679</v>
-      </c>
-      <c r="E126" s="3" t="s">
-        <v>542</v>
-      </c>
-      <c r="F126" s="3"/>
-      <c r="G126" s="3" t="s">
-        <v>757</v>
-      </c>
-      <c r="H126" s="3" t="s">
-        <v>529</v>
-      </c>
-      <c r="I126" s="3" t="s">
-        <v>530</v>
-      </c>
-      <c r="J126" s="6" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=chantal.taillon@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="127" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A127" s="5" t="s">
-        <v>531</v>
-      </c>
-      <c r="B127" s="5" t="s">
-        <v>532</v>
-      </c>
-      <c r="C127" s="5" t="s">
-        <v>533</v>
-      </c>
-      <c r="D127" s="5" t="s">
-        <v>683</v>
-      </c>
-      <c r="E127" s="5" t="s">
-        <v>76</v>
-      </c>
-      <c r="G127" s="5" t="s">
-        <v>305</v>
-      </c>
-      <c r="H127" s="5" t="s">
-        <v>534</v>
-      </c>
-      <c r="I127" s="15" t="s">
-        <v>535</v>
+      <c r="H127" t="s">
+        <v>645</v>
+      </c>
+      <c r="I127" s="6" t="s">
+        <v>646</v>
       </c>
       <c r="J127" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=mathieu.nicolas.tardif@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="128" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A128" t="s">
-        <v>644</v>
-      </c>
-      <c r="B128" t="s">
-        <v>566</v>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=nancy.theberge.2@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="128" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A128" s="5" t="s">
+        <v>536</v>
+      </c>
+      <c r="B128" s="5" t="s">
+        <v>537</v>
       </c>
       <c r="C128" s="5" t="s">
-        <v>647</v>
+        <v>614</v>
       </c>
       <c r="D128" s="5" t="s">
         <v>678</v>
       </c>
       <c r="E128" s="5"/>
-      <c r="F128" s="3"/>
-      <c r="G128" t="s">
-        <v>525</v>
-      </c>
-      <c r="H128" t="s">
-        <v>645</v>
-      </c>
-      <c r="I128" s="6" t="s">
-        <v>646</v>
+      <c r="F128" s="5"/>
+      <c r="G128" s="5" t="s">
+        <v>418</v>
+      </c>
+      <c r="H128" s="5" t="s">
+        <v>739</v>
+      </c>
+      <c r="I128" s="8" t="s">
+        <v>538</v>
       </c>
       <c r="J128" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=nancy.theberge.2@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="129" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A129" s="5" t="s">
-        <v>536</v>
-      </c>
-      <c r="B129" s="5" t="s">
-        <v>537</v>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=karine.theriault-dube@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="129" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A129" s="3" t="s">
+        <v>539</v>
+      </c>
+      <c r="B129" s="3" t="s">
+        <v>540</v>
       </c>
       <c r="C129" s="5" t="s">
-        <v>614</v>
-      </c>
-      <c r="D129" s="5" t="s">
+        <v>541</v>
+      </c>
+      <c r="D129" s="3" t="s">
+        <v>266</v>
+      </c>
+      <c r="E129" t="s">
+        <v>542</v>
+      </c>
+      <c r="F129" s="3" t="s">
+        <v>543</v>
+      </c>
+      <c r="G129" s="3" t="s">
+        <v>595</v>
+      </c>
+      <c r="H129" s="3" t="s">
+        <v>544</v>
+      </c>
+      <c r="I129" s="15" t="s">
+        <v>545</v>
+      </c>
+      <c r="J129" s="6" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=mylene.therrien@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="130" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A130" s="5" t="s">
+        <v>546</v>
+      </c>
+      <c r="B130" s="5" t="s">
+        <v>448</v>
+      </c>
+      <c r="C130" s="5" t="s">
+        <v>547</v>
+      </c>
+      <c r="D130" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="E130" s="5"/>
+      <c r="F130" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="G130" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="H130" s="5" t="s">
+        <v>548</v>
+      </c>
+      <c r="I130" s="15" t="s">
+        <v>549</v>
+      </c>
+      <c r="J130" s="6" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=m.thomas@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="131" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A131" s="5" t="s">
+        <v>550</v>
+      </c>
+      <c r="B131" s="5" t="s">
+        <v>551</v>
+      </c>
+      <c r="C131" s="5" t="s">
+        <v>627</v>
+      </c>
+      <c r="D131" s="5" t="s">
         <v>678</v>
       </c>
-      <c r="E129" s="5"/>
-      <c r="F129" s="5"/>
-      <c r="G129" s="5" t="s">
+      <c r="E131" s="5"/>
+      <c r="F131" s="5"/>
+      <c r="G131" s="5" t="s">
         <v>418</v>
       </c>
-      <c r="H129" s="5" t="s">
-        <v>742</v>
-      </c>
-      <c r="I129" s="8" t="s">
-        <v>538</v>
-      </c>
-      <c r="J129" s="6" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=karine.theriault-dube@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="130" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A130" s="3" t="s">
-        <v>539</v>
-      </c>
-      <c r="B130" s="3" t="s">
-        <v>540</v>
-      </c>
-      <c r="C130" s="5" t="s">
-        <v>541</v>
-      </c>
-      <c r="D130" s="3" t="s">
-        <v>266</v>
-      </c>
-      <c r="E130" t="s">
-        <v>542</v>
-      </c>
-      <c r="F130" s="3" t="s">
-        <v>543</v>
-      </c>
-      <c r="G130" s="3" t="s">
-        <v>595</v>
-      </c>
-      <c r="H130" s="3" t="s">
-        <v>544</v>
-      </c>
-      <c r="I130" s="15" t="s">
-        <v>545</v>
-      </c>
-      <c r="J130" s="6" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=mylene.therrien@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="131" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A131" s="5" t="s">
-        <v>546</v>
-      </c>
-      <c r="B131" s="5" t="s">
-        <v>448</v>
-      </c>
-      <c r="C131" s="5" t="s">
-        <v>547</v>
-      </c>
-      <c r="D131" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="E131" s="5"/>
-      <c r="F131" s="5" t="s">
-        <v>124</v>
-      </c>
-      <c r="G131" s="5" t="s">
-        <v>125</v>
-      </c>
-      <c r="H131" s="5" t="s">
-        <v>548</v>
-      </c>
-      <c r="I131" s="15" t="s">
-        <v>549</v>
+      <c r="H131" t="s">
+        <v>552</v>
+      </c>
+      <c r="I131" s="8" t="s">
+        <v>553</v>
       </c>
       <c r="J131" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=m.thomas@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="132" spans="1:10" x14ac:dyDescent="0.25">
+        <v>https://teams.microsoft.com/l/chat/0/0?users=ly.kieng.tir@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="132" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A132" s="5" t="s">
-        <v>550</v>
+        <v>554</v>
       </c>
       <c r="B132" s="5" t="s">
-        <v>551</v>
+        <v>555</v>
       </c>
       <c r="C132" s="5" t="s">
-        <v>627</v>
+        <v>605</v>
       </c>
       <c r="D132" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="E132" s="5"/>
+      <c r="F132" s="5" t="s">
+        <v>556</v>
+      </c>
+      <c r="G132" s="5" t="s">
+        <v>218</v>
+      </c>
+      <c r="H132" s="5" t="s">
+        <v>557</v>
+      </c>
+      <c r="I132" s="15" t="s">
+        <v>558</v>
+      </c>
+      <c r="J132" s="6" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=juliette.tirard-collet@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="133" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A133" t="s">
+        <v>559</v>
+      </c>
+      <c r="B133" t="s">
+        <v>562</v>
+      </c>
+      <c r="D133" s="5" t="s">
         <v>678</v>
       </c>
-      <c r="E132" s="5"/>
-      <c r="F132" s="5"/>
-      <c r="G132" s="5" t="s">
-        <v>418</v>
-      </c>
-      <c r="H132" t="s">
-        <v>552</v>
-      </c>
-      <c r="I132" s="8" t="s">
-        <v>553</v>
-      </c>
-      <c r="J132" s="6" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=ly.kieng.tir@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="133" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A133" s="5" t="s">
-        <v>554</v>
-      </c>
-      <c r="B133" s="5" t="s">
-        <v>555</v>
-      </c>
-      <c r="C133" s="5" t="s">
-        <v>605</v>
-      </c>
-      <c r="D133" s="5" t="s">
-        <v>101</v>
-      </c>
-      <c r="E133" s="5"/>
-      <c r="F133" s="5" t="s">
-        <v>556</v>
-      </c>
-      <c r="G133" s="5" t="s">
-        <v>218</v>
+      <c r="G133" t="s">
+        <v>284</v>
       </c>
       <c r="H133" s="5" t="s">
-        <v>557</v>
-      </c>
-      <c r="I133" s="15" t="s">
-        <v>558</v>
+        <v>563</v>
+      </c>
+      <c r="I133" s="8" t="s">
+        <v>564</v>
       </c>
       <c r="J133" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=juliette.tirard-collet@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="134" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A134" t="s">
+        <v>https://teams.microsoft.com/l/chat/0/0?users=anne-julie.tremblay.2@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="134" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A134" s="5" t="s">
         <v>559</v>
       </c>
-      <c r="B134" t="s">
-        <v>562</v>
+      <c r="B134" s="5" t="s">
+        <v>560</v>
+      </c>
+      <c r="C134" s="5" t="s">
+        <v>607</v>
       </c>
       <c r="D134" s="5" t="s">
         <v>678</v>
       </c>
-      <c r="G134" t="s">
-        <v>284</v>
+      <c r="E134" s="5"/>
+      <c r="F134" s="5"/>
+      <c r="G134" s="5" t="s">
+        <v>403</v>
       </c>
       <c r="H134" s="5" t="s">
-        <v>563</v>
+        <v>404</v>
       </c>
       <c r="I134" s="8" t="s">
-        <v>564</v>
+        <v>561</v>
       </c>
       <c r="J134" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=anne-julie.tremblay.2@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="135" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A135" s="5" t="s">
-        <v>559</v>
-      </c>
-      <c r="B135" s="5" t="s">
-        <v>560</v>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=frederic.tremblay.1@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="135" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A135" t="s">
+        <v>585</v>
+      </c>
+      <c r="B135" t="s">
+        <v>466</v>
       </c>
       <c r="C135" s="5" t="s">
-        <v>607</v>
+        <v>626</v>
       </c>
       <c r="D135" s="5" t="s">
+        <v>683</v>
+      </c>
+      <c r="E135" s="5" t="s">
+        <v>542</v>
+      </c>
+      <c r="F135" t="s">
+        <v>379</v>
+      </c>
+      <c r="G135" t="s">
+        <v>597</v>
+      </c>
+      <c r="H135" t="s">
+        <v>586</v>
+      </c>
+      <c r="I135" s="6" t="s">
+        <v>587</v>
+      </c>
+      <c r="J135" s="6" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=j.trepanier@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="136" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A136" s="5" t="s">
+        <v>565</v>
+      </c>
+      <c r="B136" s="5" t="s">
+        <v>566</v>
+      </c>
+      <c r="C136" s="5"/>
+      <c r="D136" s="5" t="s">
         <v>678</v>
       </c>
-      <c r="E135" s="5"/>
-      <c r="F135" s="5"/>
-      <c r="G135" s="5" t="s">
-        <v>403</v>
-      </c>
-      <c r="H135" s="5" t="s">
-        <v>404</v>
-      </c>
-      <c r="I135" s="8" t="s">
-        <v>561</v>
-      </c>
-      <c r="J135" s="6" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=frederic.tremblay.1@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="136" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A136" t="s">
-        <v>585</v>
-      </c>
-      <c r="B136" t="s">
-        <v>466</v>
-      </c>
-      <c r="C136" s="5" t="s">
-        <v>626</v>
-      </c>
-      <c r="D136" s="5" t="s">
-        <v>683</v>
-      </c>
-      <c r="E136" s="5" t="s">
-        <v>542</v>
-      </c>
-      <c r="F136" t="s">
-        <v>379</v>
-      </c>
-      <c r="G136" t="s">
-        <v>597</v>
-      </c>
-      <c r="H136" t="s">
-        <v>586</v>
-      </c>
-      <c r="I136" s="6" t="s">
-        <v>587</v>
+      <c r="E136" s="5"/>
+      <c r="F136" s="5"/>
+      <c r="G136" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="H136" s="5" t="s">
+        <v>567</v>
+      </c>
+      <c r="I136" s="8" t="s">
+        <v>568</v>
       </c>
       <c r="J136" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=j.trepanier@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="137" spans="1:10" x14ac:dyDescent="0.25">
+        <v>https://teams.microsoft.com/l/chat/0/0?users=nancy.turgeon@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="137" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A137" s="5" t="s">
-        <v>565</v>
+        <v>569</v>
       </c>
       <c r="B137" s="5" t="s">
-        <v>566</v>
-      </c>
-      <c r="C137" s="5"/>
+        <v>570</v>
+      </c>
+      <c r="C137" s="5" t="s">
+        <v>590</v>
+      </c>
       <c r="D137" s="5" t="s">
         <v>678</v>
       </c>
       <c r="E137" s="5"/>
       <c r="F137" s="5"/>
       <c r="G137" s="5" t="s">
-        <v>52</v>
+        <v>29</v>
       </c>
       <c r="H137" s="5" t="s">
-        <v>567</v>
+        <v>571</v>
       </c>
       <c r="I137" s="8" t="s">
-        <v>568</v>
+        <v>572</v>
       </c>
       <c r="J137" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=nancy.turgeon@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="138" spans="1:10" x14ac:dyDescent="0.25">
+        <v>https://teams.microsoft.com/l/chat/0/0?users=josee.vachon.1@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="138" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A138" s="5" t="s">
-        <v>569</v>
+        <v>573</v>
       </c>
       <c r="B138" s="5" t="s">
-        <v>570</v>
+        <v>574</v>
       </c>
       <c r="C138" s="5" t="s">
-        <v>590</v>
+        <v>616</v>
       </c>
       <c r="D138" s="5" t="s">
         <v>678</v>
@@ -7126,160 +7088,131 @@
       <c r="E138" s="5"/>
       <c r="F138" s="5"/>
       <c r="G138" s="5" t="s">
-        <v>29</v>
+        <v>52</v>
       </c>
       <c r="H138" s="5" t="s">
-        <v>571</v>
+        <v>575</v>
       </c>
       <c r="I138" s="8" t="s">
-        <v>572</v>
+        <v>576</v>
       </c>
       <c r="J138" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=josee.vachon.1@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="139" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A139" s="5" t="s">
-        <v>573</v>
-      </c>
-      <c r="B139" s="5" t="s">
-        <v>574</v>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=yan.vallee@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="139" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A139" t="s">
+        <v>713</v>
+      </c>
+      <c r="B139" t="s">
+        <v>714</v>
       </c>
       <c r="C139" s="5" t="s">
-        <v>616</v>
-      </c>
-      <c r="D139" s="5" t="s">
+        <v>726</v>
+      </c>
+      <c r="D139" t="s">
+        <v>725</v>
+      </c>
+      <c r="E139" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="G139" t="s">
+        <v>77</v>
+      </c>
+      <c r="I139" s="6" t="s">
+        <v>715</v>
+      </c>
+      <c r="J139" s="9" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=guillaume.viart@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="140" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A140" s="5" t="s">
+        <v>577</v>
+      </c>
+      <c r="B140" s="5" t="s">
+        <v>570</v>
+      </c>
+      <c r="C140" s="5" t="s">
+        <v>624</v>
+      </c>
+      <c r="D140" s="5" t="s">
         <v>678</v>
       </c>
-      <c r="E139" s="5"/>
-      <c r="F139" s="5"/>
-      <c r="G139" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="H139" s="5" t="s">
-        <v>575</v>
-      </c>
-      <c r="I139" s="8" t="s">
-        <v>576</v>
-      </c>
-      <c r="J139" s="6" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=yan.vallee@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="140" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A140" t="s">
-        <v>716</v>
-      </c>
-      <c r="B140" t="s">
-        <v>717</v>
-      </c>
-      <c r="C140" s="5" t="s">
-        <v>729</v>
-      </c>
-      <c r="D140" t="s">
-        <v>728</v>
-      </c>
-      <c r="E140" s="5" t="s">
-        <v>76</v>
-      </c>
-      <c r="G140" t="s">
-        <v>77</v>
-      </c>
-      <c r="I140" s="6" t="s">
-        <v>718</v>
-      </c>
-      <c r="J140" s="9" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=guillaume.viart@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="141" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="E140" s="5"/>
+      <c r="F140" s="5"/>
+      <c r="G140" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="H140" s="5" t="s">
+        <v>578</v>
+      </c>
+      <c r="I140" s="8" t="s">
+        <v>579</v>
+      </c>
+      <c r="J140" s="6" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=josee.viel@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="141" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A141" s="5" t="s">
-        <v>577</v>
+        <v>580</v>
       </c>
       <c r="B141" s="5" t="s">
-        <v>570</v>
-      </c>
-      <c r="C141" s="5" t="s">
-        <v>624</v>
-      </c>
+        <v>210</v>
+      </c>
+      <c r="C141" s="5"/>
       <c r="D141" s="5" t="s">
-        <v>678</v>
-      </c>
-      <c r="E141" s="5"/>
-      <c r="F141" s="5"/>
-      <c r="G141" s="5" t="s">
-        <v>87</v>
+        <v>27</v>
+      </c>
+      <c r="E141" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="F141" s="5" t="s">
+        <v>748</v>
+      </c>
+      <c r="G141" t="s">
+        <v>424</v>
       </c>
       <c r="H141" s="5" t="s">
-        <v>578</v>
-      </c>
-      <c r="I141" s="8" t="s">
-        <v>579</v>
+        <v>445</v>
+      </c>
+      <c r="I141" s="15" t="s">
+        <v>581</v>
       </c>
       <c r="J141" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=josee.viel@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="142" spans="1:10" x14ac:dyDescent="0.25">
+        <v>https://teams.microsoft.com/l/chat/0/0?users=emilie.walsh@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="142" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A142" s="5" t="s">
-        <v>580</v>
+        <v>663</v>
       </c>
       <c r="B142" s="5" t="s">
-        <v>210</v>
+        <v>664</v>
       </c>
       <c r="C142" s="5"/>
       <c r="D142" s="5" t="s">
-        <v>27</v>
+        <v>686</v>
       </c>
       <c r="E142" s="5" t="s">
-        <v>69</v>
-      </c>
-      <c r="F142" s="5" t="s">
-        <v>751</v>
-      </c>
-      <c r="G142" t="s">
-        <v>424</v>
+        <v>76</v>
+      </c>
+      <c r="F142" s="5"/>
+      <c r="G142" s="5" t="s">
+        <v>76</v>
       </c>
       <c r="H142" s="5" t="s">
-        <v>445</v>
-      </c>
-      <c r="I142" s="15" t="s">
-        <v>581</v>
-      </c>
-      <c r="J142" s="6" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=emilie.walsh@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="143" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A143" s="5" t="s">
-        <v>663</v>
-      </c>
-      <c r="B143" s="5" t="s">
-        <v>664</v>
-      </c>
-      <c r="C143" s="5"/>
-      <c r="D143" s="5" t="s">
-        <v>686</v>
-      </c>
-      <c r="E143" s="5" t="s">
-        <v>76</v>
-      </c>
-      <c r="F143" s="5"/>
-      <c r="G143" s="5" t="s">
-        <v>76</v>
-      </c>
-      <c r="H143" s="5" t="s">
         <v>665</v>
       </c>
-      <c r="I143" s="6" t="s">
+      <c r="I142" s="6" t="s">
         <v>666</v>
       </c>
-      <c r="J143" s="9" t="str">
+      <c r="J142" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=sosthene.yamale@umontreal.ca</v>
       </c>
@@ -7296,9 +7229,9 @@
     <hyperlink ref="I5" r:id="rId7" display="mailto:nadege.arsa@bib.umontreal.ca" xr:uid="{408AF5A3-35ED-4BF5-92B9-1B21C0C475D9}"/>
     <hyperlink ref="I21" r:id="rId8" display="mailto:simon.blais.longtin@umontreal.ca" xr:uid="{EA917AC7-9087-435B-A6E7-3AE1885514AA}"/>
     <hyperlink ref="I94" r:id="rId9" xr:uid="{8ABC26E9-CF81-491C-8A28-B209E6620D2A}"/>
-    <hyperlink ref="I138" r:id="rId10" xr:uid="{B455CC78-8572-42C6-950F-67FBEC488BBE}"/>
+    <hyperlink ref="I137" r:id="rId10" xr:uid="{B455CC78-8572-42C6-950F-67FBEC488BBE}"/>
     <hyperlink ref="I38" r:id="rId11" xr:uid="{7D21070C-9A14-48DF-982E-D995A034BDAD}"/>
-    <hyperlink ref="I134" r:id="rId12" xr:uid="{0C92A93F-14B9-4EBD-9C0E-42EDAA49F3AB}"/>
+    <hyperlink ref="I133" r:id="rId12" xr:uid="{0C92A93F-14B9-4EBD-9C0E-42EDAA49F3AB}"/>
     <hyperlink ref="I75" r:id="rId13" xr:uid="{DCABBE8B-8789-4957-9A88-F8585AD53BBC}"/>
     <hyperlink ref="I115" r:id="rId14" xr:uid="{C37D08E3-EE29-4008-958D-7BCCC40EBCA4}"/>
     <hyperlink ref="I52" r:id="rId15" xr:uid="{1383A46C-5C1D-4621-B4BC-67AD012D7CF5}"/>
@@ -7312,37 +7245,37 @@
     <hyperlink ref="I66" r:id="rId23" xr:uid="{6E82D57D-36A4-4928-AD91-BE73FFC7C389}"/>
     <hyperlink ref="I85" r:id="rId24" xr:uid="{278FDD6D-245D-42BB-9DC6-1D47D17CC5FD}"/>
     <hyperlink ref="I103" r:id="rId25" xr:uid="{5BCD15FE-E90C-4C6C-864A-F66215BE8839}"/>
-    <hyperlink ref="I135" r:id="rId26" xr:uid="{FDD0DDC4-7A67-4339-BDFC-3AA7CBFB9040}"/>
+    <hyperlink ref="I134" r:id="rId26" xr:uid="{FDD0DDC4-7A67-4339-BDFC-3AA7CBFB9040}"/>
     <hyperlink ref="I92" r:id="rId27" xr:uid="{6C259D22-E49F-4548-B971-5B79C0A1D1A3}"/>
     <hyperlink ref="I93" r:id="rId28" xr:uid="{7328D0A7-0B9F-4556-BBCF-C84267E93A32}"/>
     <hyperlink ref="I98" r:id="rId29" xr:uid="{7F7A355D-E6B8-443A-AF2B-0A53F4B15B21}"/>
     <hyperlink ref="I114" r:id="rId30" xr:uid="{3078ED0B-307C-47F2-B4E5-65F31B4FF7CB}"/>
-    <hyperlink ref="I129" r:id="rId31" xr:uid="{1A3BB298-F78B-474C-A8E7-739C762F9819}"/>
-    <hyperlink ref="I132" r:id="rId32" xr:uid="{9037CA9B-E8A7-4F4D-8F0A-7DD7E74AD41B}"/>
-    <hyperlink ref="I137" r:id="rId33" xr:uid="{B083C43A-D8A2-4E8E-9E8A-BDC13AA93D54}"/>
-    <hyperlink ref="I139" r:id="rId34" xr:uid="{A0852ED6-2CA4-4FFA-94EF-8EB908CD7BEB}"/>
-    <hyperlink ref="I141" r:id="rId35" xr:uid="{00BAEA16-152E-416E-A034-87CB2800061D}"/>
+    <hyperlink ref="I128" r:id="rId31" xr:uid="{1A3BB298-F78B-474C-A8E7-739C762F9819}"/>
+    <hyperlink ref="I131" r:id="rId32" xr:uid="{9037CA9B-E8A7-4F4D-8F0A-7DD7E74AD41B}"/>
+    <hyperlink ref="I136" r:id="rId33" xr:uid="{B083C43A-D8A2-4E8E-9E8A-BDC13AA93D54}"/>
+    <hyperlink ref="I138" r:id="rId34" xr:uid="{A0852ED6-2CA4-4FFA-94EF-8EB908CD7BEB}"/>
+    <hyperlink ref="I140" r:id="rId35" xr:uid="{00BAEA16-152E-416E-A034-87CB2800061D}"/>
     <hyperlink ref="I17" r:id="rId36" xr:uid="{E26D4CB1-6F14-4277-AD54-18A052872B6B}"/>
-    <hyperlink ref="I136" r:id="rId37" xr:uid="{37C73F8E-25A1-477F-AA74-E9785B7E918A}"/>
+    <hyperlink ref="I135" r:id="rId37" xr:uid="{37C73F8E-25A1-477F-AA74-E9785B7E918A}"/>
     <hyperlink ref="I40" r:id="rId38" xr:uid="{902A8808-023C-4EA1-833E-F687288B12ED}"/>
-    <hyperlink ref="I128" r:id="rId39" xr:uid="{0F562F25-AF6E-412E-962D-4CACCF0BD4F0}"/>
-    <hyperlink ref="I119" r:id="rId40" xr:uid="{349E580E-212A-42D9-8F7B-BDF3DFB61650}"/>
+    <hyperlink ref="I127" r:id="rId39" xr:uid="{0F562F25-AF6E-412E-962D-4CACCF0BD4F0}"/>
+    <hyperlink ref="I118" r:id="rId40" xr:uid="{349E580E-212A-42D9-8F7B-BDF3DFB61650}"/>
     <hyperlink ref="I54" r:id="rId41" xr:uid="{ABEB73EB-E336-4619-ADE1-0AE567E81306}"/>
     <hyperlink ref="I32" r:id="rId42" xr:uid="{E819F1D0-ED89-4281-B222-20D0A6AC8A49}"/>
-    <hyperlink ref="I143" r:id="rId43" xr:uid="{EDD92A66-A56B-419B-967E-B8D761D72C58}"/>
+    <hyperlink ref="I142" r:id="rId43" xr:uid="{EDD92A66-A56B-419B-967E-B8D761D72C58}"/>
     <hyperlink ref="I20" r:id="rId44" xr:uid="{A4113BC8-FD33-4D47-854C-D964ED926E7F}"/>
     <hyperlink ref="I116" r:id="rId45" xr:uid="{0924E3CD-F2EB-4646-BC88-767228D5A8FD}"/>
     <hyperlink ref="I76" r:id="rId46" xr:uid="{FAC375AB-8F54-402B-A4F5-618AA479650B}"/>
     <hyperlink ref="I4" r:id="rId47" xr:uid="{12EFBBCC-308A-4E41-92F6-4E78BB9E9458}"/>
     <hyperlink ref="I22" r:id="rId48" xr:uid="{CAA07608-BC3B-468C-819E-F94EE0396C78}"/>
-    <hyperlink ref="I140" r:id="rId49" xr:uid="{B3DF72B2-3730-4A9C-8195-E5B8FCD87C3B}"/>
-    <hyperlink ref="I121" r:id="rId50" xr:uid="{518A2404-8625-4373-BDE5-E73718B1440B}"/>
+    <hyperlink ref="I139" r:id="rId49" xr:uid="{B3DF72B2-3730-4A9C-8195-E5B8FCD87C3B}"/>
+    <hyperlink ref="I120" r:id="rId50" xr:uid="{518A2404-8625-4373-BDE5-E73718B1440B}"/>
     <hyperlink ref="I34" r:id="rId51" xr:uid="{B383F9BF-E7F0-4AFA-A217-1F3A922E55BA}"/>
-    <hyperlink ref="I142" r:id="rId52" xr:uid="{D2BBF900-A9C8-4032-A387-C01245244DE0}"/>
+    <hyperlink ref="I141" r:id="rId52" xr:uid="{D2BBF900-A9C8-4032-A387-C01245244DE0}"/>
     <hyperlink ref="I53" r:id="rId53" xr:uid="{79C702A2-295C-4D37-BA6F-DD2C408C75BD}"/>
     <hyperlink ref="I24" r:id="rId54" xr:uid="{761F418D-12C5-4F41-8071-6031B8FBF83B}"/>
     <hyperlink ref="I107" r:id="rId55" xr:uid="{C91A1DE6-A8FA-4481-9E51-1DB52F17F3CC}"/>
-    <hyperlink ref="I133" r:id="rId56" xr:uid="{131478F3-61ED-4B04-9E66-6F771D0E53F1}"/>
+    <hyperlink ref="I132" r:id="rId56" xr:uid="{131478F3-61ED-4B04-9E66-6F771D0E53F1}"/>
     <hyperlink ref="I101" r:id="rId57" xr:uid="{C3534DCE-62CB-4016-B559-AE879ED29221}"/>
     <hyperlink ref="I73" r:id="rId58" xr:uid="{598291DC-2DD2-464C-A65A-36D0759E8852}"/>
     <hyperlink ref="I65" r:id="rId59" xr:uid="{55FAFEEC-7E6A-4254-BBB4-020FD859DB23}"/>
@@ -7353,15 +7286,15 @@
     <hyperlink ref="I113" r:id="rId64" xr:uid="{99B099F4-5E98-4B25-B2EB-EE4C451DC6EE}"/>
     <hyperlink ref="I60" r:id="rId65" xr:uid="{1C080271-6DB7-4810-99C8-8FF2BA5EA430}"/>
     <hyperlink ref="I64" r:id="rId66" xr:uid="{6A0B0BD3-8872-437B-9CD4-6D8D7D98A4F9}"/>
-    <hyperlink ref="I122" r:id="rId67" xr:uid="{CE8C2C5F-3292-4BA9-A27E-19AF9661C907}"/>
+    <hyperlink ref="I121" r:id="rId67" xr:uid="{CE8C2C5F-3292-4BA9-A27E-19AF9661C907}"/>
     <hyperlink ref="I11" r:id="rId68" xr:uid="{F1246003-4D15-4FC5-9F7D-6CE88CAF21A8}"/>
-    <hyperlink ref="I131" r:id="rId69" xr:uid="{BB3A0149-0DD5-481B-8662-8134BB3FCECC}"/>
-    <hyperlink ref="I127" r:id="rId70" xr:uid="{52D55C85-F393-43A8-95EF-F57618BB179E}"/>
+    <hyperlink ref="I130" r:id="rId69" xr:uid="{BB3A0149-0DD5-481B-8662-8134BB3FCECC}"/>
+    <hyperlink ref="I126" r:id="rId70" xr:uid="{52D55C85-F393-43A8-95EF-F57618BB179E}"/>
     <hyperlink ref="I88" r:id="rId71" xr:uid="{CAB4CB00-83BC-4384-BF0E-208B7456F243}"/>
     <hyperlink ref="I96" r:id="rId72" xr:uid="{4B80B43B-B062-42B6-A1CE-F4CE03CDED46}"/>
     <hyperlink ref="I8" r:id="rId73" xr:uid="{BC76BE28-D367-49FE-95A3-98BB93483999}"/>
     <hyperlink ref="I48" r:id="rId74" xr:uid="{8598B756-3A70-45A7-ABB5-3EDBEF50BAF4}"/>
-    <hyperlink ref="I130" r:id="rId75" xr:uid="{07544A5C-3F38-40A4-9945-4E56F5EFFCF4}"/>
+    <hyperlink ref="I129" r:id="rId75" xr:uid="{07544A5C-3F38-40A4-9945-4E56F5EFFCF4}"/>
     <hyperlink ref="I28" r:id="rId76" xr:uid="{C341566A-DC48-4D81-91C1-E1CD275F4D60}"/>
     <hyperlink ref="I13" r:id="rId77" xr:uid="{FAAE6B3B-3F31-452F-868E-B6C650D083E8}"/>
     <hyperlink ref="I81" r:id="rId78" xr:uid="{09E37274-D8A2-4A0B-832A-E187D6213477}"/>
@@ -7389,6 +7322,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100CC83367596A4B94585FCDD3502D89912" ma:contentTypeVersion="11" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="4e4efa8c0f0f722bbfc4a6b86077b9b4">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="7c5d7804-4d0b-4e60-9ce8-4dcaa1999ed1" xmlns:ns3="9cb1c2f4-2737-4134-a1af-8acbe3d02830" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="81c6aeae46cd0fb81a99420a9570330b" ns2:_="" ns3:_="">
     <xsd:import namespace="7c5d7804-4d0b-4e60-9ce8-4dcaa1999ed1"/>
@@ -7583,15 +7525,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DBEF5B7A-066E-4CFA-AECB-2B495BA6263D}">
   <ds:schemaRefs>
@@ -7610,6 +7543,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3747C807-31DC-4949-A88C-18B7D05A7D8F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FCCC2BCD-0310-4A3C-9E4B-6EFDEBA53649}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -7626,12 +7567,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3747C807-31DC-4949-A88C-18B7D05A7D8F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>